<commit_message>
chore: update data 2026-03-17
</commit_message>
<xml_diff>
--- a/data/downloads/KY/_6VisionFeeSchedule.xlsx
+++ b/data/downloads/KY/_6VisionFeeSchedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kymsoffice-my.sharepoint.com/personal/andrea_clay_ky_gov1/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{AD58A06B-B756-4A82-9439-8E4EEE94906D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F65D2D49-97AF-42D0-9EF7-D003B272D3DE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4E5AA3B-21D6-4A29-B7C8-F63F16400F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,9 +17,9 @@
     <sheet name="Updates" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vision Fee Schedule'!$A$15:$G$266</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">Updates!$A$1:$C$17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Vision Fee Schedule'!$A$1:$G$289</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vision Fee Schedule'!$A$15:$G$267</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">Updates!$A$1:$C$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Vision Fee Schedule'!$A$1:$G$290</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Vision Fee Schedule'!$15:$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="437">
   <si>
     <t xml:space="preserve">Notes: 									</t>
   </si>
@@ -1552,21 +1552,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">KY Medicaid Vision Fee Schedule 2026  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>revised 3.6.2026</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Update to Note section to remove prior authorization requirement and include updated verbiage and expectations: </t>
     </r>
     <r>
@@ -1578,6 +1563,53 @@
         <scheme val="minor"/>
       </rPr>
       <t>More than one (1) pair of eyeglasses per recipient per calendar year – provider must keep documentation in members record stating reason a 2nd pair is required for auditing purposes.  Must meet criteria in regulation 907 KAR 1:631</t>
+    </r>
+  </si>
+  <si>
+    <t>92288</t>
+  </si>
+  <si>
+    <t>SCREENING EVALUATION OF EYE ADAPTATION TO LIGHT AND DARK WITH INTERPRETATION AND REPORT</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Code Expansion:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 92288 added to allow for a more detailed break down of description between codes 92284 and 92288. Codes 92284 and 92288 can't be billed in conjunction.</t>
+    </r>
+  </si>
+  <si>
+    <t>adult and children Effective 1/1/2026</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">KY Medicaid Vision Fee Schedule 2026  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>revised 3.17.2026</t>
     </r>
   </si>
 </sst>
@@ -1901,7 +1933,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -2040,6 +2072,24 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="23" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2048,6 +2098,12 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="21" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="34" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="34" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="23" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2063,15 +2119,6 @@
     </xf>
     <xf numFmtId="14" fontId="15" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="34" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="34" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="35">
@@ -2521,9 +2568,13 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2FA41A53-A08F-4C88-8A9D-16FF1DF1D76F}" name="Table1" displayName="Table1" ref="A15:G289" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7">
-  <autoFilter ref="A15:G289" xr:uid="{2FA41A53-A08F-4C88-8A9D-16FF1DF1D76F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2FA41A53-A08F-4C88-8A9D-16FF1DF1D76F}" name="Table1" displayName="Table1" ref="A15:G290" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7">
+  <autoFilter ref="A15:G290" xr:uid="{2FA41A53-A08F-4C88-8A9D-16FF1DF1D76F}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{3324294E-A11A-407C-B907-0EAED04C82A1}" name="Procedure_x000a_Code" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{1121C07D-3575-4C14-A188-C280D768A30C}" name="Modifier" dataDxfId="5"/>
@@ -2824,7 +2875,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G289"/>
+  <dimension ref="A1:G290"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.6640625" style="2" bestFit="1" customWidth="1"/>
@@ -2839,158 +2890,158 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="46" t="s">
-        <v>431</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
+      <c r="A1" s="52" t="s">
+        <v>436</v>
+      </c>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
     </row>
     <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
     </row>
     <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="54" t="s">
         <v>153</v>
       </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
     </row>
     <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="60" t="s">
         <v>172</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
+      <c r="B4" s="60"/>
+      <c r="C4" s="60"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="60"/>
+      <c r="G4" s="60"/>
     </row>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="59" t="s">
         <v>404</v>
       </c>
-      <c r="B5" s="51"/>
-      <c r="C5" s="51"/>
-      <c r="D5" s="51"/>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
-      <c r="G5" s="51"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
     </row>
     <row r="6" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="51" t="s">
+      <c r="A6" s="59" t="s">
         <v>418</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="59"/>
+      <c r="G6" s="59"/>
     </row>
     <row r="7" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="51" t="s">
+      <c r="A7" s="59" t="s">
         <v>157</v>
       </c>
-      <c r="B7" s="51"/>
-      <c r="C7" s="51"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="51"/>
-      <c r="G7" s="51"/>
+      <c r="B7" s="59"/>
+      <c r="C7" s="59"/>
+      <c r="D7" s="59"/>
+      <c r="E7" s="59"/>
+      <c r="F7" s="59"/>
+      <c r="G7" s="59"/>
     </row>
     <row r="8" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="51" t="s">
+      <c r="A8" s="59" t="s">
         <v>424</v>
       </c>
-      <c r="B8" s="51"/>
-      <c r="C8" s="51"/>
-      <c r="D8" s="51"/>
-      <c r="E8" s="51"/>
-      <c r="F8" s="51"/>
-      <c r="G8" s="51"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="59"/>
+      <c r="D8" s="59"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="59"/>
     </row>
     <row r="9" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="49" t="s">
+      <c r="A9" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="49"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="49"/>
+      <c r="B9" s="57"/>
+      <c r="C9" s="57"/>
+      <c r="D9" s="57"/>
+      <c r="E9" s="57"/>
+      <c r="F9" s="57"/>
+      <c r="G9" s="57"/>
     </row>
     <row r="10" spans="1:7" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="55" t="s">
         <v>430</v>
       </c>
-      <c r="B10" s="54"/>
-      <c r="C10" s="54"/>
-      <c r="D10" s="54"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="54"/>
-      <c r="G10" s="54"/>
+      <c r="B10" s="56"/>
+      <c r="C10" s="56"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="56"/>
+      <c r="F10" s="56"/>
+      <c r="G10" s="56"/>
     </row>
     <row r="11" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="50" t="s">
+      <c r="A11" s="58" t="s">
         <v>423</v>
       </c>
-      <c r="B11" s="50"/>
-      <c r="C11" s="50"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="50"/>
-      <c r="G11" s="50"/>
+      <c r="B11" s="58"/>
+      <c r="C11" s="58"/>
+      <c r="D11" s="58"/>
+      <c r="E11" s="58"/>
+      <c r="F11" s="58"/>
+      <c r="G11" s="58"/>
     </row>
     <row r="12" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="58" t="s">
         <v>425</v>
       </c>
-      <c r="B12" s="50"/>
-      <c r="C12" s="50"/>
-      <c r="D12" s="50"/>
-      <c r="E12" s="50"/>
-      <c r="F12" s="50"/>
-      <c r="G12" s="50"/>
+      <c r="B12" s="58"/>
+      <c r="C12" s="58"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="58"/>
+      <c r="F12" s="58"/>
+      <c r="G12" s="58"/>
     </row>
     <row r="13" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="50" t="s">
+      <c r="A13" s="58" t="s">
         <v>152</v>
       </c>
-      <c r="B13" s="50"/>
-      <c r="C13" s="50"/>
-      <c r="D13" s="50"/>
-      <c r="E13" s="50"/>
-      <c r="F13" s="50"/>
-      <c r="G13" s="50"/>
+      <c r="B13" s="58"/>
+      <c r="C13" s="58"/>
+      <c r="D13" s="58"/>
+      <c r="E13" s="58"/>
+      <c r="F13" s="58"/>
+      <c r="G13" s="58"/>
     </row>
     <row r="14" spans="1:7" ht="15" x14ac:dyDescent="0.2">
-      <c r="A14" s="49" t="s">
+      <c r="A14" s="57" t="s">
         <v>428</v>
       </c>
-      <c r="B14" s="49"/>
-      <c r="C14" s="49"/>
-      <c r="D14" s="49"/>
-      <c r="E14" s="49"/>
-      <c r="F14" s="49"/>
-      <c r="G14" s="49"/>
+      <c r="B14" s="57"/>
+      <c r="C14" s="57"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="57"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="57"/>
     </row>
     <row r="15" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="37" t="s">
@@ -5304,203 +5355,201 @@
         <v>156</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A137" s="17">
-        <v>92310</v>
-      </c>
-      <c r="B137" s="17"/>
-      <c r="C137" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="D137" s="14">
-        <v>69.739999999999995</v>
-      </c>
-      <c r="E137" s="14">
-        <v>69.739999999999995</v>
-      </c>
-      <c r="F137" s="14"/>
-      <c r="G137" s="5" t="s">
-        <v>156</v>
+    <row r="137" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A137" s="47" t="s">
+        <v>432</v>
+      </c>
+      <c r="B137" s="48"/>
+      <c r="C137" s="45" t="s">
+        <v>433</v>
+      </c>
+      <c r="D137" s="49">
+        <v>19.29</v>
+      </c>
+      <c r="E137" s="49">
+        <v>19.29</v>
+      </c>
+      <c r="F137" s="50"/>
+      <c r="G137" s="51" t="s">
+        <v>435</v>
       </c>
     </row>
     <row r="138" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A138" s="17">
-        <v>92311</v>
+        <v>92310</v>
       </c>
       <c r="B138" s="17"/>
       <c r="C138" s="9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D138" s="14">
-        <v>44.49</v>
+        <v>69.739999999999995</v>
       </c>
       <c r="E138" s="14">
-        <v>56.56</v>
+        <v>69.739999999999995</v>
       </c>
       <c r="F138" s="14"/>
       <c r="G138" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A139" s="6">
+    <row r="139" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A139" s="17">
+        <v>92311</v>
+      </c>
+      <c r="B139" s="17"/>
+      <c r="C139" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D139" s="14">
+        <v>44.49</v>
+      </c>
+      <c r="E139" s="14">
+        <v>56.56</v>
+      </c>
+      <c r="F139" s="14"/>
+      <c r="G139" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A140" s="6">
         <v>92312</v>
-      </c>
-      <c r="B139" s="6"/>
-      <c r="C139" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="D139" s="10">
-        <v>53.26</v>
-      </c>
-      <c r="E139" s="10">
-        <v>68.819999999999993</v>
-      </c>
-      <c r="F139" s="10"/>
-      <c r="G139" s="5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="140" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A140" s="6">
-        <v>92313</v>
       </c>
       <c r="B140" s="6"/>
       <c r="C140" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D140" s="10">
-        <v>39.53</v>
+        <v>53.26</v>
       </c>
       <c r="E140" s="10">
-        <v>51.33</v>
+        <v>68.819999999999993</v>
       </c>
       <c r="F140" s="10"/>
       <c r="G140" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A141" s="6">
-        <v>92314</v>
+        <v>92313</v>
       </c>
       <c r="B141" s="6"/>
       <c r="C141" s="9" t="s">
-        <v>400</v>
+        <v>145</v>
       </c>
       <c r="D141" s="10">
-        <v>41.17</v>
+        <v>39.53</v>
       </c>
       <c r="E141" s="10">
-        <v>41.17</v>
-      </c>
-      <c r="F141" s="10">
-        <v>41.17</v>
-      </c>
+        <v>51.33</v>
+      </c>
+      <c r="F141" s="10"/>
       <c r="G141" s="5" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="142" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A142" s="6">
-        <v>92340</v>
+        <v>92314</v>
       </c>
       <c r="B142" s="6"/>
       <c r="C142" s="9" t="s">
-        <v>146</v>
+        <v>400</v>
       </c>
       <c r="D142" s="10">
-        <v>33</v>
+        <v>41.17</v>
       </c>
       <c r="E142" s="10">
-        <v>33</v>
+        <v>41.17</v>
       </c>
       <c r="F142" s="10">
-        <v>33</v>
+        <v>41.17</v>
       </c>
       <c r="G142" s="5" t="s">
-        <v>402</v>
+        <v>156</v>
       </c>
     </row>
     <row r="143" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A143" s="6">
-        <v>92341</v>
+        <v>92340</v>
       </c>
       <c r="B143" s="6"/>
       <c r="C143" s="9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D143" s="10">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E143" s="10">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F143" s="10">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="G143" s="5" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="144" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A144" s="6">
-        <v>92342</v>
+        <v>92341</v>
       </c>
       <c r="B144" s="6"/>
       <c r="C144" s="9" t="s">
-        <v>399</v>
+        <v>147</v>
       </c>
       <c r="D144" s="10">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E144" s="10">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F144" s="10">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G144" s="5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A145" s="6">
-        <v>92352</v>
+        <v>92342</v>
       </c>
       <c r="B145" s="6"/>
       <c r="C145" s="9" t="s">
-        <v>148</v>
+        <v>399</v>
       </c>
       <c r="D145" s="10">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="E145" s="10">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F145" s="10">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="G145" s="5" t="s">
-        <v>402</v>
+        <v>156</v>
       </c>
     </row>
     <row r="146" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A146" s="6">
-        <v>92353</v>
+        <v>92352</v>
       </c>
       <c r="B146" s="6"/>
       <c r="C146" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D146" s="10">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="E146" s="10">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F146" s="10">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G146" s="5" t="s">
         <v>402</v>
@@ -5508,20 +5557,20 @@
     </row>
     <row r="147" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A147" s="6">
-        <v>92370</v>
+        <v>92353</v>
       </c>
       <c r="B147" s="6"/>
       <c r="C147" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D147" s="10">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="E147" s="10">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="F147" s="10">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="G147" s="5" t="s">
         <v>402</v>
@@ -5529,43 +5578,41 @@
     </row>
     <row r="148" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A148" s="6">
-        <v>92371</v>
+        <v>92370</v>
       </c>
       <c r="B148" s="6"/>
       <c r="C148" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D148" s="10">
+        <v>29</v>
+      </c>
+      <c r="E148" s="10">
+        <v>29</v>
+      </c>
+      <c r="F148" s="10">
+        <v>29</v>
+      </c>
+      <c r="G148" s="5" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A149" s="6">
+        <v>92371</v>
+      </c>
+      <c r="B149" s="6"/>
+      <c r="C149" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="D148" s="10">
+      <c r="D149" s="10">
         <v>8.4</v>
       </c>
-      <c r="E148" s="10">
+      <c r="E149" s="10">
         <v>16.309999999999999</v>
       </c>
-      <c r="F148" s="10" t="s">
+      <c r="F149" s="10" t="s">
         <v>81</v>
-      </c>
-      <c r="G148" s="5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A149" s="6">
-        <v>92499</v>
-      </c>
-      <c r="B149" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C149" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="D149" s="10">
-        <v>14</v>
-      </c>
-      <c r="E149" s="10">
-        <v>14</v>
-      </c>
-      <c r="F149" s="10">
-        <v>14</v>
       </c>
       <c r="G149" s="5" t="s">
         <v>156</v>
@@ -5576,19 +5623,19 @@
         <v>92499</v>
       </c>
       <c r="B150" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C150" s="9" t="s">
         <v>253</v>
       </c>
       <c r="D150" s="10">
-        <v>3.5</v>
+        <v>14</v>
       </c>
       <c r="E150" s="10">
-        <v>3.5</v>
+        <v>14</v>
       </c>
       <c r="F150" s="10">
-        <v>3.5</v>
+        <v>14</v>
       </c>
       <c r="G150" s="5" t="s">
         <v>156</v>
@@ -5596,36 +5643,40 @@
     </row>
     <row r="151" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A151" s="6">
-        <v>92531</v>
-      </c>
-      <c r="B151" s="6"/>
+        <v>92499</v>
+      </c>
+      <c r="B151" s="6" t="s">
+        <v>80</v>
+      </c>
       <c r="C151" s="9" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D151" s="10">
-        <v>6.96</v>
+        <v>3.5</v>
       </c>
       <c r="E151" s="10">
-        <v>6.96</v>
-      </c>
-      <c r="F151" s="10"/>
+        <v>3.5</v>
+      </c>
+      <c r="F151" s="10">
+        <v>3.5</v>
+      </c>
       <c r="G151" s="5" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="152" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A152" s="6">
-        <v>92532</v>
+        <v>92531</v>
       </c>
       <c r="B152" s="6"/>
       <c r="C152" s="9" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D152" s="10">
-        <v>5.83</v>
+        <v>6.96</v>
       </c>
       <c r="E152" s="10">
-        <v>5.83</v>
+        <v>6.96</v>
       </c>
       <c r="F152" s="10"/>
       <c r="G152" s="5" t="s">
@@ -5634,17 +5685,17 @@
     </row>
     <row r="153" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A153" s="6">
-        <v>92533</v>
+        <v>92532</v>
       </c>
       <c r="B153" s="6"/>
       <c r="C153" s="9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D153" s="10">
-        <v>6.69</v>
+        <v>5.83</v>
       </c>
       <c r="E153" s="10">
-        <v>6.69</v>
+        <v>5.83</v>
       </c>
       <c r="F153" s="10"/>
       <c r="G153" s="5" t="s">
@@ -5653,17 +5704,17 @@
     </row>
     <row r="154" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A154" s="6">
-        <v>92534</v>
+        <v>92533</v>
       </c>
       <c r="B154" s="6"/>
       <c r="C154" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D154" s="10">
-        <v>2.76</v>
+        <v>6.69</v>
       </c>
       <c r="E154" s="10">
-        <v>2.76</v>
+        <v>6.69</v>
       </c>
       <c r="F154" s="10"/>
       <c r="G154" s="5" t="s">
@@ -5672,112 +5723,112 @@
     </row>
     <row r="155" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A155" s="6">
-        <v>92541</v>
+        <v>92534</v>
       </c>
       <c r="B155" s="6"/>
       <c r="C155" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D155" s="10">
-        <v>31.41</v>
+        <v>2.76</v>
       </c>
       <c r="E155" s="10">
-        <v>31.41</v>
+        <v>2.76</v>
       </c>
       <c r="F155" s="10"/>
       <c r="G155" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="156" spans="1:7" s="27" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A156" s="6">
-        <v>92542</v>
+        <v>92541</v>
       </c>
       <c r="B156" s="6"/>
       <c r="C156" s="9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D156" s="10">
-        <v>27.75</v>
+        <v>31.41</v>
       </c>
       <c r="E156" s="10">
-        <v>27.75</v>
+        <v>31.41</v>
       </c>
       <c r="F156" s="10"/>
       <c r="G156" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="157" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:7" s="27" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A157" s="6">
-        <v>92544</v>
+        <v>92542</v>
       </c>
       <c r="B157" s="6"/>
       <c r="C157" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D157" s="10">
-        <v>21.45</v>
+        <v>27.75</v>
       </c>
       <c r="E157" s="10">
-        <v>21.45</v>
+        <v>27.75</v>
       </c>
       <c r="F157" s="10"/>
       <c r="G157" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="158" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A158" s="6">
-        <v>92545</v>
+        <v>92544</v>
       </c>
       <c r="B158" s="6"/>
       <c r="C158" s="9" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D158" s="10">
-        <v>18.45</v>
+        <v>21.45</v>
       </c>
       <c r="E158" s="10">
-        <v>18.45</v>
+        <v>21.45</v>
       </c>
       <c r="F158" s="10"/>
       <c r="G158" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="159" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A159" s="6">
-        <v>92546</v>
+        <v>92545</v>
       </c>
       <c r="B159" s="6"/>
       <c r="C159" s="9" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D159" s="10">
-        <v>23.94</v>
+        <v>18.45</v>
       </c>
       <c r="E159" s="10">
-        <v>23.94</v>
+        <v>18.45</v>
       </c>
       <c r="F159" s="10"/>
       <c r="G159" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="160" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A160" s="6">
-        <v>92547</v>
+        <v>92546</v>
       </c>
       <c r="B160" s="6"/>
       <c r="C160" s="9" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D160" s="10">
-        <v>15.67</v>
+        <v>23.94</v>
       </c>
       <c r="E160" s="10">
-        <v>15.67</v>
+        <v>23.94</v>
       </c>
       <c r="F160" s="10"/>
       <c r="G160" s="5" t="s">
@@ -5786,36 +5837,36 @@
     </row>
     <row r="161" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A161" s="6">
-        <v>93886</v>
+        <v>92547</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="9" t="s">
-        <v>370</v>
+        <v>263</v>
       </c>
       <c r="D161" s="10">
-        <v>158.82</v>
+        <v>15.67</v>
       </c>
       <c r="E161" s="10">
-        <v>158.82</v>
+        <v>15.67</v>
       </c>
       <c r="F161" s="10"/>
       <c r="G161" s="5" t="s">
-        <v>406</v>
+        <v>156</v>
       </c>
     </row>
     <row r="162" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A162" s="6">
-        <v>93888</v>
+        <v>93886</v>
       </c>
       <c r="B162" s="6"/>
       <c r="C162" s="9" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="D162" s="10">
-        <v>105.85</v>
+        <v>158.82</v>
       </c>
       <c r="E162" s="10">
-        <v>105.85</v>
+        <v>158.82</v>
       </c>
       <c r="F162" s="10"/>
       <c r="G162" s="5" t="s">
@@ -5824,55 +5875,55 @@
     </row>
     <row r="163" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A163" s="6">
-        <v>93892</v>
+        <v>93888</v>
       </c>
       <c r="B163" s="6"/>
       <c r="C163" s="9" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D163" s="10">
-        <v>177.44</v>
+        <v>105.85</v>
       </c>
       <c r="E163" s="10">
-        <v>177.44</v>
+        <v>105.85</v>
       </c>
       <c r="F163" s="10"/>
       <c r="G163" s="5" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="164" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A164" s="6">
-        <v>94010</v>
+        <v>93892</v>
       </c>
       <c r="B164" s="6"/>
       <c r="C164" s="9" t="s">
-        <v>264</v>
+        <v>371</v>
       </c>
       <c r="D164" s="10">
-        <v>24.44</v>
+        <v>177.44</v>
       </c>
       <c r="E164" s="10">
-        <v>24.44</v>
+        <v>177.44</v>
       </c>
       <c r="F164" s="10"/>
       <c r="G164" s="5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="165" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A165" s="6">
-        <v>95060</v>
+        <v>94010</v>
       </c>
       <c r="B165" s="6"/>
       <c r="C165" s="9" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D165" s="10">
-        <v>9.34</v>
+        <v>24.44</v>
       </c>
       <c r="E165" s="10">
-        <v>9.34</v>
+        <v>24.44</v>
       </c>
       <c r="F165" s="10"/>
       <c r="G165" s="5" t="s">
@@ -5881,93 +5932,93 @@
     </row>
     <row r="166" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A166" s="6">
-        <v>95930</v>
+        <v>95060</v>
       </c>
       <c r="B166" s="6"/>
       <c r="C166" s="9" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D166" s="10">
-        <v>33.75</v>
+        <v>9.34</v>
       </c>
       <c r="E166" s="10">
-        <v>33.75</v>
+        <v>9.34</v>
       </c>
       <c r="F166" s="10"/>
       <c r="G166" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="167" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A167" s="6">
-        <v>96112</v>
+        <v>95930</v>
       </c>
       <c r="B167" s="6"/>
       <c r="C167" s="9" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D167" s="10">
-        <v>108.86</v>
+        <v>33.75</v>
       </c>
       <c r="E167" s="10">
-        <v>108.86</v>
+        <v>33.75</v>
       </c>
       <c r="F167" s="10"/>
       <c r="G167" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="168" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A168" s="6">
-        <v>96113</v>
+        <v>96112</v>
       </c>
       <c r="B168" s="6"/>
       <c r="C168" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D168" s="10">
-        <v>48.65</v>
+        <v>108.86</v>
       </c>
       <c r="E168" s="10">
-        <v>48.65</v>
+        <v>108.86</v>
       </c>
       <c r="F168" s="10"/>
       <c r="G168" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="169" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A169" s="6">
-        <v>96116</v>
+        <v>96113</v>
       </c>
       <c r="B169" s="6"/>
       <c r="C169" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D169" s="10">
-        <v>76.180000000000007</v>
+        <v>48.65</v>
       </c>
       <c r="E169" s="10">
-        <v>81.03</v>
+        <v>48.65</v>
       </c>
       <c r="F169" s="10"/>
       <c r="G169" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="170" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A170" s="6">
-        <v>97110</v>
+        <v>96116</v>
       </c>
       <c r="B170" s="6"/>
       <c r="C170" s="9" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D170" s="10">
-        <v>20.9</v>
+        <v>76.180000000000007</v>
       </c>
       <c r="E170" s="10">
-        <v>20.9</v>
+        <v>81.03</v>
       </c>
       <c r="F170" s="10"/>
       <c r="G170" s="5" t="s">
@@ -5976,36 +6027,36 @@
     </row>
     <row r="171" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A171" s="6">
-        <v>97112</v>
+        <v>97110</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D171" s="10">
-        <v>21.66</v>
+        <v>20.9</v>
       </c>
       <c r="E171" s="10">
-        <v>21.66</v>
+        <v>20.9</v>
       </c>
       <c r="F171" s="10"/>
       <c r="G171" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="172" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A172" s="6">
-        <v>97150</v>
+        <v>97112</v>
       </c>
       <c r="B172" s="6"/>
       <c r="C172" s="9" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D172" s="10">
-        <v>13.77</v>
+        <v>21.66</v>
       </c>
       <c r="E172" s="10">
-        <v>13.77</v>
+        <v>21.66</v>
       </c>
       <c r="F172" s="10"/>
       <c r="G172" s="5" t="s">
@@ -6014,55 +6065,55 @@
     </row>
     <row r="173" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A173" s="6">
-        <v>97530</v>
+        <v>97150</v>
       </c>
       <c r="B173" s="6"/>
       <c r="C173" s="9" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D173" s="10">
-        <v>21.61</v>
+        <v>13.77</v>
       </c>
       <c r="E173" s="10">
-        <v>21.61</v>
+        <v>13.77</v>
       </c>
       <c r="F173" s="10"/>
       <c r="G173" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="174" spans="1:7" ht="114.75" x14ac:dyDescent="0.2">
-      <c r="A174" s="33" t="s">
-        <v>167</v>
+    <row r="174" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A174" s="6">
+        <v>97530</v>
       </c>
       <c r="B174" s="6"/>
-      <c r="C174" s="34" t="s">
-        <v>411</v>
-      </c>
-      <c r="D174" s="35">
-        <v>22.53</v>
-      </c>
-      <c r="E174" s="35">
-        <v>22.53</v>
+      <c r="C174" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="D174" s="10">
+        <v>21.61</v>
+      </c>
+      <c r="E174" s="10">
+        <v>21.61</v>
       </c>
       <c r="F174" s="10"/>
-      <c r="G174" s="34" t="s">
-        <v>170</v>
+      <c r="G174" s="5" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="175" spans="1:7" ht="114.75" x14ac:dyDescent="0.2">
       <c r="A175" s="33" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B175" s="6"/>
       <c r="C175" s="34" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D175" s="35">
-        <v>10.88</v>
+        <v>22.53</v>
       </c>
       <c r="E175" s="35">
-        <v>10.88</v>
+        <v>22.53</v>
       </c>
       <c r="F175" s="10"/>
       <c r="G175" s="34" t="s">
@@ -6071,74 +6122,74 @@
     </row>
     <row r="176" spans="1:7" ht="114.75" x14ac:dyDescent="0.2">
       <c r="A176" s="33" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="34" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="D176" s="35">
-        <v>8.0299999999999994</v>
+        <v>10.88</v>
       </c>
       <c r="E176" s="35">
-        <v>8.0299999999999994</v>
+        <v>10.88</v>
       </c>
       <c r="F176" s="10"/>
       <c r="G176" s="34" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="177" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A177" s="6">
+    <row r="177" spans="1:7" ht="114.75" x14ac:dyDescent="0.2">
+      <c r="A177" s="33" t="s">
+        <v>169</v>
+      </c>
+      <c r="B177" s="6"/>
+      <c r="C177" s="34" t="s">
+        <v>413</v>
+      </c>
+      <c r="D177" s="35">
+        <v>8.0299999999999994</v>
+      </c>
+      <c r="E177" s="35">
+        <v>8.0299999999999994</v>
+      </c>
+      <c r="F177" s="10"/>
+      <c r="G177" s="34" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A178" s="6">
         <v>99050</v>
-      </c>
-      <c r="B177" s="6"/>
-      <c r="C177" s="9" t="s">
-        <v>274</v>
-      </c>
-      <c r="D177" s="10">
-        <v>7.5</v>
-      </c>
-      <c r="E177" s="10">
-        <v>10</v>
-      </c>
-      <c r="F177" s="10"/>
-      <c r="G177" s="5" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="178" spans="1:7" ht="89.25" x14ac:dyDescent="0.2">
-      <c r="A178" s="6">
-        <v>99202</v>
       </c>
       <c r="B178" s="6"/>
       <c r="C178" s="9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D178" s="10">
-        <v>39.729999999999997</v>
+        <v>7.5</v>
       </c>
       <c r="E178" s="10">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="F178" s="10"/>
       <c r="G178" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="179" spans="1:7" ht="89.25" x14ac:dyDescent="0.2">
       <c r="A179" s="6">
-        <v>99203</v>
+        <v>99202</v>
       </c>
       <c r="B179" s="6"/>
       <c r="C179" s="9" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D179" s="10">
-        <v>60.57</v>
+        <v>39.729999999999997</v>
       </c>
       <c r="E179" s="10">
-        <v>79.040000000000006</v>
+        <v>53</v>
       </c>
       <c r="F179" s="10"/>
       <c r="G179" s="5" t="s">
@@ -6147,17 +6198,17 @@
     </row>
     <row r="180" spans="1:7" ht="89.25" x14ac:dyDescent="0.2">
       <c r="A180" s="6">
-        <v>99204</v>
+        <v>99203</v>
       </c>
       <c r="B180" s="6"/>
       <c r="C180" s="9" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D180" s="10">
-        <v>102.79</v>
+        <v>60.57</v>
       </c>
       <c r="E180" s="10">
-        <v>112.27</v>
+        <v>79.040000000000006</v>
       </c>
       <c r="F180" s="10"/>
       <c r="G180" s="5" t="s">
@@ -6166,150 +6217,150 @@
     </row>
     <row r="181" spans="1:7" ht="89.25" x14ac:dyDescent="0.2">
       <c r="A181" s="6">
-        <v>99205</v>
+        <v>99204</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="9" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D181" s="10">
-        <v>131.97999999999999</v>
+        <v>102.79</v>
       </c>
       <c r="E181" s="10">
-        <v>143.29</v>
+        <v>112.27</v>
       </c>
       <c r="F181" s="10"/>
       <c r="G181" s="5" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="182" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:7" ht="89.25" x14ac:dyDescent="0.2">
       <c r="A182" s="6">
-        <v>99211</v>
+        <v>99205</v>
       </c>
       <c r="B182" s="6"/>
       <c r="C182" s="9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D182" s="10">
-        <v>7.48</v>
+        <v>131.97999999999999</v>
       </c>
       <c r="E182" s="10">
-        <v>16.98</v>
+        <v>143.29</v>
       </c>
       <c r="F182" s="10"/>
       <c r="G182" s="5" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="183" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A183" s="6">
-        <v>99212</v>
+        <v>99211</v>
       </c>
       <c r="B183" s="6"/>
       <c r="C183" s="9" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D183" s="10">
-        <v>20.41</v>
+        <v>7.48</v>
       </c>
       <c r="E183" s="10">
-        <v>31.08</v>
+        <v>16.98</v>
       </c>
       <c r="F183" s="10"/>
       <c r="G183" s="5" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="184" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A184" s="6">
-        <v>99213</v>
+        <v>99212</v>
       </c>
       <c r="B184" s="6"/>
       <c r="C184" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D184" s="10">
-        <v>40.36</v>
+        <v>20.41</v>
       </c>
       <c r="E184" s="10">
-        <v>42.63</v>
+        <v>31.08</v>
       </c>
       <c r="F184" s="10"/>
       <c r="G184" s="5" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="185" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A185" s="6">
-        <v>99214</v>
+        <v>99213</v>
       </c>
       <c r="B185" s="6"/>
       <c r="C185" s="9" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D185" s="10">
-        <v>61.98</v>
+        <v>40.36</v>
       </c>
       <c r="E185" s="10">
-        <v>67.099999999999994</v>
+        <v>42.63</v>
       </c>
       <c r="F185" s="10"/>
       <c r="G185" s="5" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="186" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A186" s="6">
-        <v>99215</v>
+        <v>99214</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="9" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D186" s="10">
-        <v>87.17</v>
+        <v>61.98</v>
       </c>
       <c r="E186" s="10">
-        <v>98.39</v>
+        <v>67.099999999999994</v>
       </c>
       <c r="F186" s="10"/>
       <c r="G186" s="5" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="187" spans="1:7" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A187" s="6">
-        <v>99221</v>
+        <v>99215</v>
       </c>
       <c r="B187" s="6"/>
       <c r="C187" s="9" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D187" s="10">
-        <v>51.66</v>
+        <v>87.17</v>
       </c>
       <c r="E187" s="10">
-        <v>51.66</v>
+        <v>98.39</v>
       </c>
       <c r="F187" s="10"/>
       <c r="G187" s="5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="188" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A188" s="6">
-        <v>99222</v>
+        <v>99221</v>
       </c>
       <c r="B188" s="6"/>
       <c r="C188" s="9" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D188" s="10">
-        <v>85.6</v>
+        <v>51.66</v>
       </c>
       <c r="E188" s="10">
-        <v>85.6</v>
+        <v>51.66</v>
       </c>
       <c r="F188" s="10"/>
       <c r="G188" s="5" t="s">
@@ -6318,55 +6369,55 @@
     </row>
     <row r="189" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A189" s="6">
-        <v>99223</v>
+        <v>99222</v>
       </c>
       <c r="B189" s="6"/>
       <c r="C189" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D189" s="10">
-        <v>119.25</v>
+        <v>85.6</v>
       </c>
       <c r="E189" s="10">
-        <v>119.25</v>
+        <v>85.6</v>
       </c>
       <c r="F189" s="10"/>
       <c r="G189" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="190" spans="1:7" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A190" s="6">
-        <v>99231</v>
+        <v>99223</v>
       </c>
       <c r="B190" s="6"/>
       <c r="C190" s="9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D190" s="10">
-        <v>25.89</v>
+        <v>119.25</v>
       </c>
       <c r="E190" s="10">
-        <v>25.89</v>
+        <v>119.25</v>
       </c>
       <c r="F190" s="10"/>
       <c r="G190" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="191" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:7" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A191" s="6">
-        <v>99232</v>
+        <v>99231</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="9" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D191" s="10">
-        <v>42.24</v>
+        <v>25.89</v>
       </c>
       <c r="E191" s="10">
-        <v>42.24</v>
+        <v>25.89</v>
       </c>
       <c r="F191" s="10"/>
       <c r="G191" s="5" t="s">
@@ -6375,74 +6426,74 @@
     </row>
     <row r="192" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A192" s="6">
-        <v>99233</v>
+        <v>99232</v>
       </c>
       <c r="B192" s="6"/>
       <c r="C192" s="9" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D192" s="10">
-        <v>60.07</v>
+        <v>42.24</v>
       </c>
       <c r="E192" s="10">
-        <v>60.07</v>
+        <v>42.24</v>
       </c>
       <c r="F192" s="10"/>
       <c r="G192" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="193" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A193" s="6">
-        <v>99238</v>
+        <v>99233</v>
       </c>
       <c r="B193" s="6"/>
       <c r="C193" s="9" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D193" s="10">
-        <v>53.44</v>
+        <v>60.07</v>
       </c>
       <c r="E193" s="10">
-        <v>53.44</v>
+        <v>60.07</v>
       </c>
       <c r="F193" s="10"/>
       <c r="G193" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="194" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A194" s="6">
-        <v>99239</v>
+        <v>99238</v>
       </c>
       <c r="B194" s="6"/>
       <c r="C194" s="9" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D194" s="10">
-        <v>72.89</v>
+        <v>53.44</v>
       </c>
       <c r="E194" s="10">
-        <v>72.89</v>
+        <v>53.44</v>
       </c>
       <c r="F194" s="10"/>
       <c r="G194" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="195" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A195" s="6">
-        <v>99242</v>
+        <v>99239</v>
       </c>
       <c r="B195" s="6"/>
       <c r="C195" s="9" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D195" s="10">
-        <v>54.91</v>
+        <v>72.89</v>
       </c>
       <c r="E195" s="10">
-        <v>67.83</v>
+        <v>72.89</v>
       </c>
       <c r="F195" s="10"/>
       <c r="G195" s="5" t="s">
@@ -6451,17 +6502,17 @@
     </row>
     <row r="196" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A196" s="6">
-        <v>99243</v>
+        <v>99242</v>
       </c>
       <c r="B196" s="6"/>
       <c r="C196" s="9" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D196" s="10">
-        <v>76.53</v>
+        <v>54.91</v>
       </c>
       <c r="E196" s="10">
-        <v>90.43</v>
+        <v>67.83</v>
       </c>
       <c r="F196" s="10"/>
       <c r="G196" s="5" t="s">
@@ -6470,17 +6521,17 @@
     </row>
     <row r="197" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A197" s="6">
-        <v>99244</v>
+        <v>99243</v>
       </c>
       <c r="B197" s="6"/>
       <c r="C197" s="9" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D197" s="10">
-        <v>121.37</v>
+        <v>76.53</v>
       </c>
       <c r="E197" s="10">
-        <v>128.22</v>
+        <v>90.43</v>
       </c>
       <c r="F197" s="10"/>
       <c r="G197" s="5" t="s">
@@ -6489,17 +6540,17 @@
     </row>
     <row r="198" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A198" s="6">
-        <v>99245</v>
+        <v>99244</v>
       </c>
       <c r="B198" s="6"/>
       <c r="C198" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D198" s="10">
-        <v>150.75</v>
+        <v>121.37</v>
       </c>
       <c r="E198" s="10">
-        <v>166.18</v>
+        <v>128.22</v>
       </c>
       <c r="F198" s="10"/>
       <c r="G198" s="5" t="s">
@@ -6508,17 +6559,17 @@
     </row>
     <row r="199" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A199" s="6">
-        <v>99252</v>
+        <v>99245</v>
       </c>
       <c r="B199" s="6"/>
       <c r="C199" s="9" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D199" s="10">
-        <v>55.73</v>
+        <v>150.75</v>
       </c>
       <c r="E199" s="10">
-        <v>55.73</v>
+        <v>166.18</v>
       </c>
       <c r="F199" s="10"/>
       <c r="G199" s="5" t="s">
@@ -6527,17 +6578,17 @@
     </row>
     <row r="200" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A200" s="6">
-        <v>99253</v>
+        <v>99252</v>
       </c>
       <c r="B200" s="6"/>
       <c r="C200" s="9" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D200" s="10">
-        <v>74.75</v>
+        <v>55.73</v>
       </c>
       <c r="E200" s="10">
-        <v>74.75</v>
+        <v>55.73</v>
       </c>
       <c r="F200" s="10"/>
       <c r="G200" s="5" t="s">
@@ -6546,17 +6597,17 @@
     </row>
     <row r="201" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A201" s="6">
-        <v>99254</v>
+        <v>99253</v>
       </c>
       <c r="B201" s="6"/>
       <c r="C201" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D201" s="10">
-        <v>107.5</v>
+        <v>74.75</v>
       </c>
       <c r="E201" s="10">
-        <v>107.5</v>
+        <v>74.75</v>
       </c>
       <c r="F201" s="10"/>
       <c r="G201" s="5" t="s">
@@ -6565,74 +6616,74 @@
     </row>
     <row r="202" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A202" s="6">
-        <v>99255</v>
+        <v>99254</v>
       </c>
       <c r="B202" s="6"/>
       <c r="C202" s="9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D202" s="10">
-        <v>148.19999999999999</v>
+        <v>107.5</v>
       </c>
       <c r="E202" s="10">
-        <v>148.19999999999999</v>
+        <v>107.5</v>
       </c>
       <c r="F202" s="10"/>
       <c r="G202" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="203" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A203" s="17">
+    <row r="203" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A203" s="6">
+        <v>99255</v>
+      </c>
+      <c r="B203" s="6"/>
+      <c r="C203" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="D203" s="10">
+        <v>148.19999999999999</v>
+      </c>
+      <c r="E203" s="10">
+        <v>148.19999999999999</v>
+      </c>
+      <c r="F203" s="10"/>
+      <c r="G203" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="204" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A204" s="17">
         <v>99281</v>
       </c>
-      <c r="B203" s="17"/>
-      <c r="C203" s="9" t="s">
+      <c r="B204" s="17"/>
+      <c r="C204" s="9" t="s">
         <v>300</v>
       </c>
-      <c r="D203" s="14">
+      <c r="D204" s="14">
         <v>15.97</v>
       </c>
-      <c r="E203" s="14">
+      <c r="E204" s="14">
         <v>15.97</v>
       </c>
-      <c r="F203" s="14"/>
-      <c r="G203" s="5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="204" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A204" s="6">
-        <v>99282</v>
-      </c>
-      <c r="B204" s="6"/>
-      <c r="C204" s="9" t="s">
-        <v>301</v>
-      </c>
-      <c r="D204" s="10">
-        <v>24.71</v>
-      </c>
-      <c r="E204" s="10">
-        <v>24.71</v>
-      </c>
-      <c r="F204" s="10"/>
+      <c r="F204" s="14"/>
       <c r="G204" s="5" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="205" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A205" s="6">
-        <v>99283</v>
+        <v>99282</v>
       </c>
       <c r="B205" s="6"/>
       <c r="C205" s="9" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D205" s="10">
-        <v>47.4</v>
+        <v>24.71</v>
       </c>
       <c r="E205" s="10">
-        <v>47.4</v>
+        <v>24.71</v>
       </c>
       <c r="F205" s="10"/>
       <c r="G205" s="5" t="s">
@@ -6641,17 +6692,17 @@
     </row>
     <row r="206" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A206" s="6">
-        <v>99284</v>
+        <v>99283</v>
       </c>
       <c r="B206" s="6"/>
       <c r="C206" s="9" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D206" s="10">
-        <v>74.05</v>
+        <v>47.4</v>
       </c>
       <c r="E206" s="10">
-        <v>74.05</v>
+        <v>47.4</v>
       </c>
       <c r="F206" s="10"/>
       <c r="G206" s="5" t="s">
@@ -6660,98 +6711,100 @@
     </row>
     <row r="207" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A207" s="6">
-        <v>99285</v>
+        <v>99284</v>
       </c>
       <c r="B207" s="6"/>
       <c r="C207" s="9" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D207" s="10">
-        <v>116.04</v>
+        <v>74.05</v>
       </c>
       <c r="E207" s="10">
-        <v>116.04</v>
+        <v>74.05</v>
       </c>
       <c r="F207" s="10"/>
       <c r="G207" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="208" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A208" s="6">
-        <v>99341</v>
+        <v>99285</v>
       </c>
       <c r="B208" s="6"/>
       <c r="C208" s="9" t="s">
-        <v>305</v>
-      </c>
-      <c r="D208" s="10"/>
+        <v>304</v>
+      </c>
+      <c r="D208" s="10">
+        <v>116.04</v>
+      </c>
       <c r="E208" s="10">
-        <v>74.38</v>
+        <v>116.04</v>
       </c>
       <c r="F208" s="10"/>
       <c r="G208" s="5" t="s">
-        <v>395</v>
+        <v>156</v>
       </c>
     </row>
     <row r="209" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A209" s="6">
-        <v>99342</v>
+        <v>99341</v>
       </c>
       <c r="B209" s="6"/>
       <c r="C209" s="9" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D209" s="10"/>
       <c r="E209" s="10">
-        <v>98.05</v>
+        <v>74.38</v>
       </c>
       <c r="F209" s="10"/>
       <c r="G209" s="5" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="210" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A210" s="6">
+        <v>99342</v>
+      </c>
+      <c r="B210" s="6"/>
+      <c r="C210" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="D210" s="10"/>
+      <c r="E210" s="10">
+        <v>98.05</v>
+      </c>
+      <c r="F210" s="10"/>
+      <c r="G210" s="5" t="s">
         <v>405</v>
-      </c>
-    </row>
-    <row r="210" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A210" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B210" s="7"/>
-      <c r="C210" s="9" t="s">
-        <v>307</v>
-      </c>
-      <c r="D210" s="18"/>
-      <c r="E210" s="18"/>
-      <c r="F210" s="10">
-        <v>50</v>
-      </c>
-      <c r="G210" s="5" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="211" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A211" s="7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B211" s="7"/>
       <c r="C211" s="9" t="s">
-        <v>308</v>
-      </c>
-      <c r="D211" s="14"/>
-      <c r="E211" s="14"/>
+        <v>307</v>
+      </c>
+      <c r="D211" s="18"/>
+      <c r="E211" s="18"/>
       <c r="F211" s="10">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="G211" s="5" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="212" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="212" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A212" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B212" s="7"/>
       <c r="C212" s="9" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D212" s="14"/>
       <c r="E212" s="14"/>
@@ -6762,13 +6815,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="213" spans="1:7" s="8" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A213" s="32" t="s">
-        <v>94</v>
+    <row r="213" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A213" s="7" t="s">
+        <v>7</v>
       </c>
       <c r="B213" s="7"/>
       <c r="C213" s="9" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D213" s="14"/>
       <c r="E213" s="14"/>
@@ -6779,13 +6832,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="214" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A214" s="7" t="s">
-        <v>8</v>
+    <row r="214" spans="1:7" s="8" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A214" s="32" t="s">
+        <v>94</v>
       </c>
       <c r="B214" s="7"/>
       <c r="C214" s="9" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D214" s="14"/>
       <c r="E214" s="14"/>
@@ -6798,11 +6851,11 @@
     </row>
     <row r="215" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A215" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B215" s="7"/>
       <c r="C215" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D215" s="14"/>
       <c r="E215" s="14"/>
@@ -6815,11 +6868,11 @@
     </row>
     <row r="216" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A216" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B216" s="7"/>
       <c r="C216" s="9" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D216" s="14"/>
       <c r="E216" s="14"/>
@@ -6832,11 +6885,11 @@
     </row>
     <row r="217" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A217" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B217" s="7"/>
       <c r="C217" s="9" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D217" s="14"/>
       <c r="E217" s="14"/>
@@ -6849,11 +6902,11 @@
     </row>
     <row r="218" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A218" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B218" s="7"/>
       <c r="C218" s="9" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D218" s="14"/>
       <c r="E218" s="14"/>
@@ -6866,11 +6919,11 @@
     </row>
     <row r="219" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A219" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B219" s="7"/>
       <c r="C219" s="9" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D219" s="14"/>
       <c r="E219" s="14"/>
@@ -6883,11 +6936,11 @@
     </row>
     <row r="220" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A220" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B220" s="7"/>
       <c r="C220" s="9" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D220" s="14"/>
       <c r="E220" s="14"/>
@@ -6900,11 +6953,11 @@
     </row>
     <row r="221" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A221" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B221" s="7"/>
       <c r="C221" s="9" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D221" s="14"/>
       <c r="E221" s="14"/>
@@ -6917,11 +6970,11 @@
     </row>
     <row r="222" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A222" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B222" s="7"/>
       <c r="C222" s="9" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D222" s="14"/>
       <c r="E222" s="14"/>
@@ -6934,11 +6987,11 @@
     </row>
     <row r="223" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A223" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B223" s="7"/>
       <c r="C223" s="9" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D223" s="14"/>
       <c r="E223" s="14"/>
@@ -6951,11 +7004,11 @@
     </row>
     <row r="224" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A224" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B224" s="7"/>
       <c r="C224" s="9" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D224" s="14"/>
       <c r="E224" s="14"/>
@@ -6966,13 +7019,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="225" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A225" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B225" s="7"/>
       <c r="C225" s="9" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D225" s="14"/>
       <c r="E225" s="14"/>
@@ -6983,13 +7036,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="226" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A226" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B226" s="7"/>
       <c r="C226" s="9" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D226" s="14"/>
       <c r="E226" s="14"/>
@@ -7002,11 +7055,11 @@
     </row>
     <row r="227" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A227" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B227" s="7"/>
       <c r="C227" s="9" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D227" s="14"/>
       <c r="E227" s="14"/>
@@ -7019,11 +7072,11 @@
     </row>
     <row r="228" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A228" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B228" s="7"/>
       <c r="C228" s="9" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D228" s="14"/>
       <c r="E228" s="14"/>
@@ -7036,11 +7089,11 @@
     </row>
     <row r="229" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A229" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B229" s="7"/>
       <c r="C229" s="9" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D229" s="14"/>
       <c r="E229" s="14"/>
@@ -7053,28 +7106,28 @@
     </row>
     <row r="230" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A230" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B230" s="7"/>
       <c r="C230" s="9" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D230" s="14"/>
       <c r="E230" s="14"/>
       <c r="F230" s="10">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="G230" s="5" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="231" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A231" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B231" s="7"/>
       <c r="C231" s="9" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D231" s="14"/>
       <c r="E231" s="14"/>
@@ -7087,11 +7140,11 @@
     </row>
     <row r="232" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A232" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B232" s="7"/>
       <c r="C232" s="9" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D232" s="14"/>
       <c r="E232" s="14"/>
@@ -7104,11 +7157,11 @@
     </row>
     <row r="233" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A233" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B233" s="7"/>
       <c r="C233" s="9" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D233" s="14"/>
       <c r="E233" s="14"/>
@@ -7121,11 +7174,11 @@
     </row>
     <row r="234" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A234" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B234" s="7"/>
       <c r="C234" s="9" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D234" s="14"/>
       <c r="E234" s="14"/>
@@ -7138,11 +7191,11 @@
     </row>
     <row r="235" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A235" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B235" s="7"/>
       <c r="C235" s="9" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D235" s="14"/>
       <c r="E235" s="14"/>
@@ -7155,11 +7208,11 @@
     </row>
     <row r="236" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A236" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B236" s="7"/>
       <c r="C236" s="9" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D236" s="14"/>
       <c r="E236" s="14"/>
@@ -7170,13 +7223,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="237" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A237" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B237" s="7"/>
       <c r="C237" s="9" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D237" s="14"/>
       <c r="E237" s="14"/>
@@ -7189,11 +7242,11 @@
     </row>
     <row r="238" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A238" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B238" s="7"/>
       <c r="C238" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D238" s="14"/>
       <c r="E238" s="14"/>
@@ -7206,11 +7259,11 @@
     </row>
     <row r="239" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A239" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B239" s="7"/>
       <c r="C239" s="9" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D239" s="14"/>
       <c r="E239" s="14"/>
@@ -7223,11 +7276,11 @@
     </row>
     <row r="240" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A240" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B240" s="7"/>
       <c r="C240" s="9" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D240" s="14"/>
       <c r="E240" s="14"/>
@@ -7240,11 +7293,11 @@
     </row>
     <row r="241" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A241" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B241" s="7"/>
       <c r="C241" s="9" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D241" s="14"/>
       <c r="E241" s="14"/>
@@ -7257,11 +7310,11 @@
     </row>
     <row r="242" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A242" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B242" s="7"/>
       <c r="C242" s="9" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D242" s="14"/>
       <c r="E242" s="14"/>
@@ -7274,11 +7327,11 @@
     </row>
     <row r="243" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A243" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B243" s="7"/>
       <c r="C243" s="9" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D243" s="14"/>
       <c r="E243" s="14"/>
@@ -7289,13 +7342,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="244" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A244" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B244" s="7"/>
       <c r="C244" s="9" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D244" s="14"/>
       <c r="E244" s="14"/>
@@ -7306,13 +7359,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="245" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A245" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B245" s="7"/>
       <c r="C245" s="9" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D245" s="14"/>
       <c r="E245" s="14"/>
@@ -7325,11 +7378,11 @@
     </row>
     <row r="246" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A246" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B246" s="7"/>
       <c r="C246" s="9" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D246" s="14"/>
       <c r="E246" s="14"/>
@@ -7342,11 +7395,11 @@
     </row>
     <row r="247" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A247" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B247" s="7"/>
       <c r="C247" s="9" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D247" s="14"/>
       <c r="E247" s="14"/>
@@ -7359,11 +7412,11 @@
     </row>
     <row r="248" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A248" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B248" s="7"/>
       <c r="C248" s="9" t="s">
-        <v>77</v>
+        <v>344</v>
       </c>
       <c r="D248" s="14"/>
       <c r="E248" s="14"/>
@@ -7376,11 +7429,11 @@
     </row>
     <row r="249" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A249" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B249" s="7"/>
       <c r="C249" s="9" t="s">
-        <v>345</v>
+        <v>77</v>
       </c>
       <c r="D249" s="14"/>
       <c r="E249" s="14"/>
@@ -7393,11 +7446,11 @@
     </row>
     <row r="250" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A250" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B250" s="7"/>
       <c r="C250" s="9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D250" s="14"/>
       <c r="E250" s="14"/>
@@ -7410,28 +7463,28 @@
     </row>
     <row r="251" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A251" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B251" s="7"/>
       <c r="C251" s="9" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D251" s="14"/>
       <c r="E251" s="14"/>
       <c r="F251" s="10">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="G251" s="5" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="252" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A252" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B252" s="7"/>
       <c r="C252" s="9" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D252" s="14"/>
       <c r="E252" s="14"/>
@@ -7444,11 +7497,11 @@
     </row>
     <row r="253" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A253" s="7" t="s">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="B253" s="7"/>
       <c r="C253" s="9" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D253" s="14"/>
       <c r="E253" s="14"/>
@@ -7461,11 +7514,11 @@
     </row>
     <row r="254" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A254" s="7" t="s">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="B254" s="7"/>
       <c r="C254" s="9" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D254" s="14"/>
       <c r="E254" s="14"/>
@@ -7478,11 +7531,11 @@
     </row>
     <row r="255" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A255" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B255" s="7"/>
       <c r="C255" s="9" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D255" s="14"/>
       <c r="E255" s="14"/>
@@ -7495,11 +7548,11 @@
     </row>
     <row r="256" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A256" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B256" s="7"/>
       <c r="C256" s="9" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D256" s="14"/>
       <c r="E256" s="14"/>
@@ -7512,11 +7565,11 @@
     </row>
     <row r="257" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A257" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B257" s="7"/>
       <c r="C257" s="9" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D257" s="14"/>
       <c r="E257" s="14"/>
@@ -7527,13 +7580,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="258" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A258" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B258" s="7"/>
       <c r="C258" s="9" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D258" s="14"/>
       <c r="E258" s="14"/>
@@ -7546,11 +7599,11 @@
     </row>
     <row r="259" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A259" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B259" s="7"/>
       <c r="C259" s="9" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D259" s="14"/>
       <c r="E259" s="14"/>
@@ -7563,11 +7616,11 @@
     </row>
     <row r="260" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A260" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B260" s="7"/>
       <c r="C260" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D260" s="14"/>
       <c r="E260" s="14"/>
@@ -7580,11 +7633,11 @@
     </row>
     <row r="261" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A261" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B261" s="7"/>
       <c r="C261" s="9" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D261" s="14"/>
       <c r="E261" s="14"/>
@@ -7597,11 +7650,11 @@
     </row>
     <row r="262" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A262" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B262" s="7"/>
       <c r="C262" s="9" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D262" s="14"/>
       <c r="E262" s="14"/>
@@ -7614,11 +7667,11 @@
     </row>
     <row r="263" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A263" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B263" s="7"/>
       <c r="C263" s="9" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D263" s="14"/>
       <c r="E263" s="14"/>
@@ -7631,11 +7684,11 @@
     </row>
     <row r="264" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A264" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B264" s="7"/>
       <c r="C264" s="9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D264" s="14"/>
       <c r="E264" s="14"/>
@@ -7646,13 +7699,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="265" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A265" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B265" s="7"/>
       <c r="C265" s="9" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D265" s="14"/>
       <c r="E265" s="14"/>
@@ -7663,13 +7716,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="266" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A266" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B266" s="7"/>
       <c r="C266" s="9" t="s">
-        <v>76</v>
+        <v>361</v>
       </c>
       <c r="D266" s="14"/>
       <c r="E266" s="14"/>
@@ -7680,13 +7733,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="267" spans="1:7" s="15" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A267" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B267" s="7"/>
       <c r="C267" s="9" t="s">
-        <v>362</v>
+        <v>76</v>
       </c>
       <c r="D267" s="14"/>
       <c r="E267" s="14"/>
@@ -7699,11 +7752,11 @@
     </row>
     <row r="268" spans="1:7" s="15" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A268" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B268" s="7"/>
       <c r="C268" s="9" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D268" s="14"/>
       <c r="E268" s="14"/>
@@ -7716,11 +7769,11 @@
     </row>
     <row r="269" spans="1:7" s="15" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A269" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B269" s="7"/>
       <c r="C269" s="9" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D269" s="14"/>
       <c r="E269" s="14"/>
@@ -7731,13 +7784,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="270" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:7" s="15" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A270" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B270" s="7"/>
       <c r="C270" s="9" t="s">
-        <v>75</v>
+        <v>364</v>
       </c>
       <c r="D270" s="14"/>
       <c r="E270" s="14"/>
@@ -7750,11 +7803,11 @@
     </row>
     <row r="271" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A271" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B271" s="7"/>
       <c r="C271" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D271" s="14"/>
       <c r="E271" s="14"/>
@@ -7765,13 +7818,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="272" spans="1:7" s="8" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A272" s="32" t="s">
-        <v>95</v>
+    <row r="272" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A272" s="7" t="s">
+        <v>64</v>
       </c>
       <c r="B272" s="7"/>
       <c r="C272" s="9" t="s">
-        <v>365</v>
+        <v>74</v>
       </c>
       <c r="D272" s="14"/>
       <c r="E272" s="14"/>
@@ -7782,69 +7835,69 @@
         <v>154</v>
       </c>
     </row>
-    <row r="273" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A273" s="7" t="s">
-        <v>65</v>
+    <row r="273" spans="1:7" s="8" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A273" s="32" t="s">
+        <v>95</v>
       </c>
       <c r="B273" s="7"/>
       <c r="C273" s="9" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D273" s="14"/>
       <c r="E273" s="14"/>
       <c r="F273" s="10">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="G273" s="5" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="274" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:7" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A274" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B274" s="7"/>
       <c r="C274" s="9" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D274" s="14"/>
       <c r="E274" s="14"/>
       <c r="F274" s="10">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="G274" s="5" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="275" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A275" s="32" t="s">
-        <v>96</v>
+    <row r="275" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A275" s="7" t="s">
+        <v>66</v>
       </c>
       <c r="B275" s="7"/>
       <c r="C275" s="9" t="s">
-        <v>107</v>
+        <v>367</v>
       </c>
       <c r="D275" s="14"/>
       <c r="E275" s="14"/>
       <c r="F275" s="10">
-        <v>58.24</v>
+        <v>56</v>
       </c>
       <c r="G275" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="276" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A276" s="32" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B276" s="7"/>
       <c r="C276" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D276" s="14"/>
       <c r="E276" s="14"/>
       <c r="F276" s="10">
-        <v>90.95</v>
+        <v>58.24</v>
       </c>
       <c r="G276" s="5" t="s">
         <v>155</v>
@@ -7852,16 +7905,16 @@
     </row>
     <row r="277" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A277" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B277" s="7"/>
       <c r="C277" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D277" s="14"/>
       <c r="E277" s="14"/>
       <c r="F277" s="10">
-        <v>106.04</v>
+        <v>90.95</v>
       </c>
       <c r="G277" s="5" t="s">
         <v>155</v>
@@ -7869,16 +7922,16 @@
     </row>
     <row r="278" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A278" s="32" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B278" s="7"/>
       <c r="C278" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D278" s="14"/>
       <c r="E278" s="14"/>
       <c r="F278" s="10">
-        <v>102.58</v>
+        <v>106.04</v>
       </c>
       <c r="G278" s="5" t="s">
         <v>155</v>
@@ -7886,67 +7939,67 @@
     </row>
     <row r="279" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A279" s="32" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B279" s="7"/>
       <c r="C279" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D279" s="14"/>
       <c r="E279" s="14"/>
       <c r="F279" s="10">
-        <v>46.04</v>
+        <v>102.58</v>
       </c>
       <c r="G279" s="5" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="280" spans="1:7" s="8" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
-      <c r="A280" s="7" t="s">
-        <v>83</v>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="280" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A280" s="32" t="s">
+        <v>100</v>
       </c>
       <c r="B280" s="7"/>
       <c r="C280" s="9" t="s">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="D280" s="14"/>
       <c r="E280" s="14"/>
       <c r="F280" s="10">
-        <v>104</v>
+        <v>46.04</v>
       </c>
       <c r="G280" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="281" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A281" s="32" t="s">
-        <v>101</v>
+        <v>158</v>
+      </c>
+    </row>
+    <row r="281" spans="1:7" s="8" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A281" s="7" t="s">
+        <v>83</v>
       </c>
       <c r="B281" s="7"/>
       <c r="C281" s="9" t="s">
-        <v>112</v>
+        <v>84</v>
       </c>
       <c r="D281" s="14"/>
       <c r="E281" s="14"/>
       <c r="F281" s="10">
-        <v>26.74</v>
+        <v>104</v>
       </c>
       <c r="G281" s="5" t="s">
-        <v>158</v>
+        <v>89</v>
       </c>
     </row>
     <row r="282" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A282" s="32" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B282" s="7"/>
       <c r="C282" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D282" s="14"/>
       <c r="E282" s="14"/>
       <c r="F282" s="10">
-        <v>19.329999999999998</v>
+        <v>26.74</v>
       </c>
       <c r="G282" s="5" t="s">
         <v>158</v>
@@ -7954,16 +8007,16 @@
     </row>
     <row r="283" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A283" s="32" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="B283" s="7"/>
       <c r="C283" s="9" t="s">
-        <v>88</v>
+        <v>113</v>
       </c>
       <c r="D283" s="14"/>
       <c r="E283" s="14"/>
       <c r="F283" s="10">
-        <v>14.4</v>
+        <v>19.329999999999998</v>
       </c>
       <c r="G283" s="5" t="s">
         <v>158</v>
@@ -7971,16 +8024,16 @@
     </row>
     <row r="284" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A284" s="32" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="B284" s="7"/>
       <c r="C284" s="9" t="s">
-        <v>114</v>
+        <v>88</v>
       </c>
       <c r="D284" s="14"/>
       <c r="E284" s="14"/>
       <c r="F284" s="10">
-        <v>21.73</v>
+        <v>14.4</v>
       </c>
       <c r="G284" s="5" t="s">
         <v>158</v>
@@ -7988,92 +8041,109 @@
     </row>
     <row r="285" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A285" s="32" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B285" s="7"/>
       <c r="C285" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D285" s="14"/>
       <c r="E285" s="14"/>
       <c r="F285" s="10">
-        <v>60</v>
+        <v>21.73</v>
       </c>
       <c r="G285" s="5" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="286" spans="1:7" s="8" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:7" s="8" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A286" s="32" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B286" s="7"/>
       <c r="C286" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D286" s="14"/>
       <c r="E286" s="14"/>
       <c r="F286" s="10">
-        <v>60.41</v>
+        <v>60</v>
       </c>
       <c r="G286" s="5" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="287" spans="1:7" s="8" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:7" s="8" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A287" s="32" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B287" s="7"/>
       <c r="C287" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D287" s="14"/>
       <c r="E287" s="14"/>
       <c r="F287" s="10">
-        <v>77.14</v>
+        <v>60.41</v>
       </c>
       <c r="G287" s="5" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="288" spans="1:7" s="15" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:7" s="8" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A288" s="32" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="B288" s="7"/>
       <c r="C288" s="9" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="D288" s="14"/>
       <c r="E288" s="14"/>
       <c r="F288" s="10">
-        <v>32</v>
+        <v>77.14</v>
       </c>
       <c r="G288" s="5" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A289" s="39" t="s">
+    <row r="289" spans="1:7" s="15" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A289" s="32" t="s">
+        <v>86</v>
+      </c>
+      <c r="B289" s="7"/>
+      <c r="C289" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D289" s="14"/>
+      <c r="E289" s="14"/>
+      <c r="F289" s="10">
+        <v>32</v>
+      </c>
+      <c r="G289" s="5" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="290" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A290" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="B289" s="39"/>
-      <c r="C289" s="40" t="s">
+      <c r="B290" s="39"/>
+      <c r="C290" s="40" t="s">
         <v>118</v>
       </c>
-      <c r="D289" s="41"/>
-      <c r="E289" s="41"/>
-      <c r="F289" s="42">
+      <c r="D290" s="41"/>
+      <c r="E290" s="41"/>
+      <c r="F290" s="42">
         <v>15</v>
       </c>
-      <c r="G289" s="43" t="s">
+      <c r="G290" s="43" t="s">
         <v>119</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A16:G289">
-    <sortCondition ref="A16:A289"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A16:G290">
+    <sortCondition ref="A16:A290"/>
   </sortState>
   <mergeCells count="14">
     <mergeCell ref="A1:G1"/>
@@ -8094,7 +8164,7 @@
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.25" footer="0.25"/>
   <pageSetup scale="80" orientation="landscape" r:id="rId1"/>
   <headerFooter>
-    <oddHeader>&amp;CKentucky Medicaid Vision Fee Schedule 2026&amp;RRevised 3.6.2026</oddHeader>
+    <oddHeader>&amp;CKentucky Medicaid Vision Fee Schedule 2026&amp;RRevised 3.17.2026</oddHeader>
     <oddFooter>&amp;L&amp;9https://www.chfs.ky.gov/agencies/dms/Pages/feesrates.aspx&amp;C&amp;G&amp;R&amp;P</oddFooter>
   </headerFooter>
   <drawing r:id="rId2"/>
@@ -8105,43 +8175,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{05C60535-1F16-4fd2-B633-F4F36F0B64E0}">
       <x14:sparklineGroups xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{06046525-6968-4C6C-A84F-A6EFF62FF531}">
-          <x14:colorSeries rgb="FF376092"/>
-          <x14:colorNegative rgb="FFD00000"/>
-          <x14:colorAxis rgb="FF000000"/>
-          <x14:colorMarkers rgb="FFD00000"/>
-          <x14:colorFirst rgb="FFD00000"/>
-          <x14:colorLast rgb="FFD00000"/>
-          <x14:colorHigh rgb="FFD00000"/>
-          <x14:colorLow rgb="FFD00000"/>
-          <x14:sparklines>
-            <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$A174:$A174</xm:f>
-              <xm:sqref>A174</xm:sqref>
-            </x14:sparkline>
-          </x14:sparklines>
-        </x14:sparklineGroup>
-        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{2E885D69-206A-4483-96F7-64AD7FE47308}">
-          <x14:colorSeries rgb="FF376092"/>
-          <x14:colorNegative rgb="FFD00000"/>
-          <x14:colorAxis rgb="FF000000"/>
-          <x14:colorMarkers rgb="FFD00000"/>
-          <x14:colorFirst rgb="FFD00000"/>
-          <x14:colorLast rgb="FFD00000"/>
-          <x14:colorHigh rgb="FFD00000"/>
-          <x14:colorLow rgb="FFD00000"/>
-          <x14:sparklines>
-            <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$A175:$A175</xm:f>
-              <xm:sqref>A175</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$A176:$A176</xm:f>
-              <xm:sqref>A176</xm:sqref>
-            </x14:sparkline>
-          </x14:sparklines>
-        </x14:sparklineGroup>
-        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{6F96E9CE-CB51-433F-87D4-D3FD056B2995}">
+        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{A7E511F5-C47E-4490-BE7E-427A727D03E5}">
           <x14:colorSeries rgb="FF376092"/>
           <x14:colorNegative rgb="FFD00000"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -8157,7 +8191,7 @@
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
-        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{8437974D-51C8-4B11-B4C4-51E6514F9F62}">
+        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{02851D9B-CFE5-45BD-B86B-CD5040B416C6}">
           <x14:colorSeries rgb="FF376092"/>
           <x14:colorNegative rgb="FFD00000"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -8168,32 +8202,12 @@
           <x14:colorLow rgb="FFD00000"/>
           <x14:sparklines>
             <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$D174:$D174</xm:f>
-              <xm:sqref>D174</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$D175:$D175</xm:f>
-              <xm:sqref>D175</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$D176:$D176</xm:f>
-              <xm:sqref>D176</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$E174:$E174</xm:f>
-              <xm:sqref>E174</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$E175:$E175</xm:f>
-              <xm:sqref>E175</xm:sqref>
-            </x14:sparkline>
-            <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$E176:$E176</xm:f>
-              <xm:sqref>E176</xm:sqref>
+              <xm:f>'Vision Fee Schedule'!$B175:$B175</xm:f>
+              <xm:sqref>C175</xm:sqref>
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
-        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{F9A26BDF-51AD-47E9-8304-F0A819BE864B}">
+        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{EF049BF6-DBA0-4D02-A68D-75CAB0FC8766}">
           <x14:colorSeries rgb="FF376092"/>
           <x14:colorNegative rgb="FFD00000"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -8204,12 +8218,28 @@
           <x14:colorLow rgb="FFD00000"/>
           <x14:sparklines>
             <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$I174:$I174</xm:f>
-              <xm:sqref>G174</xm:sqref>
+              <xm:f>'Vision Fee Schedule'!$I177:$I177</xm:f>
+              <xm:sqref>G177</xm:sqref>
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
         <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{05AD597E-CDC1-4B8B-8AAA-F998BC744AE7}">
+          <x14:colorSeries rgb="FF376092"/>
+          <x14:colorNegative rgb="FFD00000"/>
+          <x14:colorAxis rgb="FF000000"/>
+          <x14:colorMarkers rgb="FFD00000"/>
+          <x14:colorFirst rgb="FFD00000"/>
+          <x14:colorLast rgb="FFD00000"/>
+          <x14:colorHigh rgb="FFD00000"/>
+          <x14:colorLow rgb="FFD00000"/>
+          <x14:sparklines>
+            <x14:sparkline>
+              <xm:f>'Vision Fee Schedule'!$I176:$I176</xm:f>
+              <xm:sqref>G176</xm:sqref>
+            </x14:sparkline>
+          </x14:sparklines>
+        </x14:sparklineGroup>
+        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{F9A26BDF-51AD-47E9-8304-F0A819BE864B}">
           <x14:colorSeries rgb="FF376092"/>
           <x14:colorNegative rgb="FFD00000"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -8225,7 +8255,7 @@
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
-        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{EF049BF6-DBA0-4D02-A68D-75CAB0FC8766}">
+        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{8437974D-51C8-4B11-B4C4-51E6514F9F62}">
           <x14:colorSeries rgb="FF376092"/>
           <x14:colorNegative rgb="FFD00000"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -8236,12 +8266,32 @@
           <x14:colorLow rgb="FFD00000"/>
           <x14:sparklines>
             <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$I176:$I176</xm:f>
-              <xm:sqref>G176</xm:sqref>
+              <xm:f>'Vision Fee Schedule'!$D175:$D175</xm:f>
+              <xm:sqref>D175</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Vision Fee Schedule'!$D176:$D176</xm:f>
+              <xm:sqref>D176</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Vision Fee Schedule'!$D177:$D177</xm:f>
+              <xm:sqref>D177</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Vision Fee Schedule'!$E175:$E175</xm:f>
+              <xm:sqref>E175</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Vision Fee Schedule'!$E176:$E176</xm:f>
+              <xm:sqref>E176</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Vision Fee Schedule'!$E177:$E177</xm:f>
+              <xm:sqref>E177</xm:sqref>
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
-        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{02851D9B-CFE5-45BD-B86B-CD5040B416C6}">
+        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{6F96E9CE-CB51-433F-87D4-D3FD056B2995}">
           <x14:colorSeries rgb="FF376092"/>
           <x14:colorNegative rgb="FFD00000"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -8252,12 +8302,12 @@
           <x14:colorLow rgb="FFD00000"/>
           <x14:sparklines>
             <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$B174:$B174</xm:f>
-              <xm:sqref>C174</xm:sqref>
+              <xm:f>'Vision Fee Schedule'!$B177:$B177</xm:f>
+              <xm:sqref>C177</xm:sqref>
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
-        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{A7E511F5-C47E-4490-BE7E-427A727D03E5}">
+        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{2E885D69-206A-4483-96F7-64AD7FE47308}">
           <x14:colorSeries rgb="FF376092"/>
           <x14:colorNegative rgb="FFD00000"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -8268,8 +8318,28 @@
           <x14:colorLow rgb="FFD00000"/>
           <x14:sparklines>
             <x14:sparkline>
-              <xm:f>'Vision Fee Schedule'!$B175:$B175</xm:f>
-              <xm:sqref>C175</xm:sqref>
+              <xm:f>'Vision Fee Schedule'!$A176:$A176</xm:f>
+              <xm:sqref>A176</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Vision Fee Schedule'!$A177:$A177</xm:f>
+              <xm:sqref>A177</xm:sqref>
+            </x14:sparkline>
+          </x14:sparklines>
+        </x14:sparklineGroup>
+        <x14:sparklineGroup manualMax="0" manualMin="0" displayEmptyCellsAs="gap" xr2:uid="{06046525-6968-4C6C-A84F-A6EFF62FF531}">
+          <x14:colorSeries rgb="FF376092"/>
+          <x14:colorNegative rgb="FFD00000"/>
+          <x14:colorAxis rgb="FF000000"/>
+          <x14:colorMarkers rgb="FFD00000"/>
+          <x14:colorFirst rgb="FFD00000"/>
+          <x14:colorLast rgb="FFD00000"/>
+          <x14:colorHigh rgb="FFD00000"/>
+          <x14:colorLow rgb="FFD00000"/>
+          <x14:sparklines>
+            <x14:sparkline>
+              <xm:f>'Vision Fee Schedule'!$A175:$A175</xm:f>
+              <xm:sqref>A175</xm:sqref>
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
@@ -8290,11 +8360,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="61" t="s">
         <v>162</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
     </row>
     <row r="2" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
@@ -8465,17 +8535,23 @@
       <c r="A17" s="25" t="s">
         <v>368</v>
       </c>
-      <c r="B17" s="56" t="s">
-        <v>432</v>
+      <c r="B17" s="46" t="s">
+        <v>431</v>
       </c>
       <c r="C17" s="24">
         <v>46087</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="25"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="25"/>
+    <row r="18" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="24">
+        <v>46023</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>434</v>
+      </c>
+      <c r="C18" s="24">
+        <v>46098</v>
+      </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="25"/>
@@ -8927,23 +9003,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Search_x0020_Year xmlns="9d98fa39-7fbd-4685-a488-797cac822720">24</Search_x0020_Year>
-    <chfsDmsFeeRateSchedTerms xmlns="fdbd306d-9ecd-4c95-826c-c285ba0bc3b3">Vision</chfsDmsFeeRateSchedTerms>
-    <b9w7 xmlns="dcdf0062-15e6-47f3-91ae-956c1b802128">2026-03-06T14:55:00+00:00</b9w7>
-    <Provider_x0020_Type xmlns="9d98fa39-7fbd-4685-a488-797cac822720">
-      <Value>35</Value>
-      <Value>91</Value>
-      <Value>70</Value>
-      <Value>3</Value>
-    </Provider_x0020_Type>
-    <Waiver_x0020_Type xmlns="9d98fa39-7fbd-4685-a488-797cac822720"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="DMS Provider Letter" ma:contentTypeID="0x0101008DA2CD0899BBAE4D907571C6908B6AC70012190DE0FAEAD649A0F28B976FB5BD99" ma:contentTypeVersion="8" ma:contentTypeDescription="" ma:contentTypeScope="" ma:versionID="479a302da38c571107451cc7528011dc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9d98fa39-7fbd-4685-a488-797cac822720" xmlns:ns3="fdbd306d-9ecd-4c95-826c-c285ba0bc3b3" xmlns:ns4="dcdf0062-15e6-47f3-91ae-956c1b802128" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5619a5c2a8808acecbb7bfd83a9ac2e3" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="9d98fa39-7fbd-4685-a488-797cac822720"/>
@@ -9162,7 +9221,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -9171,19 +9230,24 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0CAD55AF-B8B9-4FB8-BD6B-72D81231A905}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9d98fa39-7fbd-4685-a488-797cac822720"/>
-    <ds:schemaRef ds:uri="fdbd306d-9ecd-4c95-826c-c285ba0bc3b3"/>
-    <ds:schemaRef ds:uri="dcdf0062-15e6-47f3-91ae-956c1b802128"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Search_x0020_Year xmlns="9d98fa39-7fbd-4685-a488-797cac822720">24</Search_x0020_Year>
+    <chfsDmsFeeRateSchedTerms xmlns="fdbd306d-9ecd-4c95-826c-c285ba0bc3b3">Vision</chfsDmsFeeRateSchedTerms>
+    <b9w7 xmlns="dcdf0062-15e6-47f3-91ae-956c1b802128">2026-03-17T14:35:00+00:00</b9w7>
+    <Provider_x0020_Type xmlns="9d98fa39-7fbd-4685-a488-797cac822720">
+      <Value>35</Value>
+      <Value>91</Value>
+      <Value>70</Value>
+      <Value>3</Value>
+    </Provider_x0020_Type>
+    <Waiver_x0020_Type xmlns="9d98fa39-7fbd-4685-a488-797cac822720"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8223BD24-4D52-4330-A220-4C11C71CF644}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9203,10 +9267,22 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5ABD0637-C222-48FB-AFF0-482EF8553D1F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0CAD55AF-B8B9-4FB8-BD6B-72D81231A905}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9d98fa39-7fbd-4685-a488-797cac822720"/>
+    <ds:schemaRef ds:uri="fdbd306d-9ecd-4c95-826c-c285ba0bc3b3"/>
+    <ds:schemaRef ds:uri="dcdf0062-15e6-47f3-91ae-956c1b802128"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>